<commit_message>
Fix FI Total row Currency column: H → G to match item rows
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/final_invoice.xlsx
+++ b/templates/final_invoice.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rotork-my.sharepoint.com/personal/jeongtaek_bang_rotork_com/Documents/바탕 화면/업무/NOAH ACTUATION/noahAutomation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="8_{69FBBAE9-3359-454D-8387-2509559CBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C042140-9DC6-46C1-83AC-0D08300EB023}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="8_{69FBBAE9-3359-454D-8387-2509559CBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A09D2061-DE89-42FB-8DAA-F52323BDB2BC}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Rotork Controls Korea Co., Ltd.</t>
   </si>
@@ -76,9 +76,6 @@
   </si>
   <si>
     <t>EA</t>
-  </si>
-  <si>
-    <t>USD</t>
   </si>
   <si>
     <t>Full General Sales Terms Conditions can be found at</t>
@@ -525,6 +522,78 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="24" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="24" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="24" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -535,7 +604,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -546,81 +614,10 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="24" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="24" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="24" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
@@ -999,17 +996,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
+      <c r="A1" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
       <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -1025,13 +1022,13 @@
       <c r="J2" s="13"/>
     </row>
     <row r="3" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
@@ -1039,13 +1036,13 @@
       <c r="J3" s="13"/>
     </row>
     <row r="4" spans="1:10" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1053,13 +1050,13 @@
       <c r="J4" s="13"/>
     </row>
     <row r="5" spans="1:10" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
@@ -1079,35 +1076,35 @@
       <c r="J6" s="13"/>
     </row>
     <row r="7" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="40" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="40"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
+      <c r="A7" s="67" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="67"/>
+      <c r="C7" s="63"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63"/>
       <c r="F7" s="20"/>
       <c r="G7" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
+      <c r="H7" s="63"/>
+      <c r="I7" s="63"/>
       <c r="J7" s="13"/>
     </row>
     <row r="8" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="41"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
+      <c r="A8" s="68" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="68"/>
+      <c r="C8" s="55"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
       <c r="F8" s="20"/>
       <c r="G8" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="H8" s="42"/>
-      <c r="I8" s="42"/>
+      <c r="H8" s="55"/>
+      <c r="I8" s="55"/>
       <c r="J8" s="13"/>
     </row>
     <row r="9" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1120,8 +1117,8 @@
       <c r="G9" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="H9" s="42"/>
-      <c r="I9" s="42"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
       <c r="J9" s="13"/>
     </row>
     <row r="10" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1132,67 +1129,67 @@
       <c r="E10" s="19"/>
       <c r="F10" s="20"/>
       <c r="G10" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="H10" s="42"/>
-      <c r="I10" s="42"/>
+        <v>21</v>
+      </c>
+      <c r="H10" s="55"/>
+      <c r="I10" s="55"/>
       <c r="J10" s="13"/>
     </row>
     <row r="11" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E11" s="17"/>
       <c r="F11" s="25"/>
       <c r="G11" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11" s="45"/>
-      <c r="I11" s="45"/>
+        <v>18</v>
+      </c>
+      <c r="H11" s="56"/>
+      <c r="I11" s="56"/>
       <c r="J11" s="13"/>
     </row>
     <row r="12" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="42"/>
-      <c r="B12" s="42"/>
-      <c r="C12" s="42"/>
-      <c r="D12" s="42"/>
-      <c r="E12" s="42"/>
+      <c r="A12" s="55"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
       <c r="F12" s="15"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="42"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
       <c r="J12" s="13"/>
     </row>
     <row r="13" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="42"/>
-      <c r="B13" s="42"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="42"/>
+      <c r="A13" s="55"/>
+      <c r="B13" s="55"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="55"/>
       <c r="F13" s="15"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="42"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="55"/>
+      <c r="I13" s="55"/>
       <c r="J13" s="13"/>
     </row>
     <row r="14" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="42"/>
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="42"/>
+      <c r="A14" s="55"/>
+      <c r="B14" s="55"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
       <c r="F14" s="15"/>
-      <c r="G14" s="42"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="42"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
       <c r="J14" s="13"/>
     </row>
     <row r="15" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="17"/>
-      <c r="B15" s="47"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="48"/>
-      <c r="E15" s="48"/>
+      <c r="B15" s="41"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="42"/>
       <c r="F15" s="15"/>
       <c r="G15" s="19"/>
       <c r="H15" s="15"/>
@@ -1200,12 +1197,12 @@
       <c r="J15" s="13"/>
     </row>
     <row r="16" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="43" t="s">
+      <c r="A16" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="44"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="44"/>
+      <c r="B16" s="70"/>
+      <c r="C16" s="70"/>
+      <c r="D16" s="70"/>
       <c r="E16" s="29" t="s">
         <v>7</v>
       </c>
@@ -1215,103 +1212,103 @@
       <c r="G16" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="H16" s="38" t="s">
+      <c r="H16" s="65" t="s">
         <v>10</v>
       </c>
-      <c r="I16" s="39"/>
+      <c r="I16" s="66"/>
       <c r="J16" s="13"/>
     </row>
     <row r="17" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="57"/>
-      <c r="B17" s="58"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="58"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="61"/>
-      <c r="H17" s="62"/>
-      <c r="I17" s="63"/>
+      <c r="A17" s="45"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="35"/>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="57"/>
-      <c r="B18" s="58"/>
-      <c r="C18" s="58"/>
-      <c r="D18" s="58"/>
-      <c r="E18" s="59"/>
-      <c r="F18" s="60"/>
-      <c r="G18" s="61"/>
-      <c r="H18" s="62"/>
-      <c r="I18" s="63"/>
+      <c r="A18" s="45"/>
+      <c r="B18" s="46"/>
+      <c r="C18" s="46"/>
+      <c r="D18" s="46"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="35"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="57"/>
-      <c r="B19" s="58"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="59"/>
-      <c r="F19" s="60"/>
-      <c r="G19" s="61"/>
-      <c r="H19" s="62"/>
-      <c r="I19" s="63"/>
+      <c r="A19" s="45"/>
+      <c r="B19" s="46"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="46"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="35"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="57"/>
-      <c r="B20" s="58"/>
-      <c r="C20" s="58"/>
-      <c r="D20" s="58"/>
-      <c r="E20" s="59"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="61"/>
-      <c r="H20" s="62"/>
-      <c r="I20" s="63"/>
+      <c r="A20" s="45"/>
+      <c r="B20" s="46"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="35"/>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="57"/>
-      <c r="B21" s="58"/>
-      <c r="C21" s="58"/>
-      <c r="D21" s="58"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="61"/>
-      <c r="H21" s="62"/>
-      <c r="I21" s="63"/>
+      <c r="A21" s="45"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="35"/>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="57"/>
-      <c r="B22" s="58"/>
-      <c r="C22" s="58"/>
-      <c r="D22" s="58"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="61"/>
-      <c r="H22" s="62"/>
-      <c r="I22" s="63"/>
+      <c r="A22" s="45"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="35"/>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="64"/>
-      <c r="B23" s="65"/>
-      <c r="C23" s="65"/>
-      <c r="D23" s="65"/>
-      <c r="E23" s="66"/>
-      <c r="F23" s="67"/>
-      <c r="G23" s="68"/>
-      <c r="H23" s="69"/>
-      <c r="I23" s="70"/>
+      <c r="A23" s="43"/>
+      <c r="B23" s="44"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="40"/>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="55" t="s">
+      <c r="A24" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="B24" s="56"/>
-      <c r="C24" s="56"/>
-      <c r="D24" s="56"/>
+      <c r="B24" s="54"/>
+      <c r="C24" s="54"/>
+      <c r="D24" s="54"/>
       <c r="E24" s="21">
         <f>SUM(E17:E23)</f>
         <v>0</v>
@@ -1320,9 +1317,7 @@
         <v>12</v>
       </c>
       <c r="G24" s="23"/>
-      <c r="H24" s="22" t="s">
-        <v>13</v>
-      </c>
+      <c r="H24" s="22"/>
       <c r="I24" s="24">
         <f>SUM(I17:I23)</f>
         <v>0</v>
@@ -1330,15 +1325,15 @@
       <c r="J24" s="2"/>
     </row>
     <row r="25" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54"/>
-      <c r="C25" s="54"/>
-      <c r="D25" s="54"/>
-      <c r="E25" s="54"/>
-      <c r="F25" s="54"/>
-      <c r="G25" s="54"/>
-      <c r="H25" s="54"/>
-      <c r="I25" s="54"/>
+      <c r="A25" s="51"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="52"/>
+      <c r="D25" s="52"/>
+      <c r="E25" s="52"/>
+      <c r="F25" s="52"/>
+      <c r="G25" s="52"/>
+      <c r="H25" s="52"/>
+      <c r="I25" s="52"/>
       <c r="J25" s="3"/>
     </row>
     <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1505,17 +1500,17 @@
       <c r="J39" s="6"/>
     </row>
     <row r="40" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="51" t="s">
-        <v>21</v>
-      </c>
-      <c r="B40" s="52"/>
-      <c r="C40" s="52"/>
-      <c r="D40" s="52"/>
-      <c r="E40" s="52"/>
-      <c r="F40" s="52"/>
-      <c r="G40" s="52"/>
-      <c r="H40" s="52"/>
-      <c r="I40" s="52"/>
+      <c r="A40" s="49" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" s="50"/>
+      <c r="C40" s="50"/>
+      <c r="D40" s="50"/>
+      <c r="E40" s="50"/>
+      <c r="F40" s="50"/>
+      <c r="G40" s="50"/>
+      <c r="H40" s="50"/>
+      <c r="I40" s="50"/>
       <c r="J40" s="6"/>
     </row>
     <row r="41" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1531,39 +1526,23 @@
       <c r="J41" s="6"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A42" s="49" t="s">
+      <c r="A42" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42" s="48"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="48"/>
+      <c r="E42" s="48"/>
+      <c r="F42" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="B42" s="50"/>
-      <c r="C42" s="50"/>
-      <c r="D42" s="50"/>
-      <c r="E42" s="50"/>
-      <c r="F42" s="46" t="s">
-        <v>15</v>
-      </c>
-      <c r="G42" s="37"/>
-      <c r="H42" s="37"/>
-      <c r="I42" s="37"/>
+      <c r="G42" s="58"/>
+      <c r="H42" s="58"/>
+      <c r="I42" s="58"/>
       <c r="J42" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A42:E42"/>
-    <mergeCell ref="A40:I40"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A25:I25"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="G12:I14"/>
-    <mergeCell ref="F42:I42"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="H7:I7"/>
@@ -1580,6 +1559,22 @@
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="G12:I14"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A20:D20"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Add Incoterms/shipping method to overseas shipping + reorder sync output
- Dashboard: add Incoterms, Shipping method columns to overseas shipping
  DN detail table and new "운송방식별 현황" summary tab
- sync_db: move summary table to end of output for better bat UX

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/final_invoice.xlsx
+++ b/templates/final_invoice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rotork-my.sharepoint.com/personal/jeongtaek_bang_rotork_com/Documents/바탕 화면/업무/NOAH ACTUATION/noahAutomation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="8_{69FBBAE9-3359-454D-8387-2509559CBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A09D2061-DE89-42FB-8DAA-F52323BDB2BC}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{69FBBAE9-3359-454D-8387-2509559CBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCF52F5D-AEA5-43B5-8871-8C05B75C44BC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -126,7 +126,7 @@
     <numFmt numFmtId="177" formatCode="#,##0.00_ "/>
     <numFmt numFmtId="178" formatCode="#,##0.00_);[Red]\(#,##0.00\)"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -291,6 +291,13 @@
       <u/>
       <sz val="8"/>
       <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -502,9 +509,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="176" fontId="17" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
@@ -534,9 +538,6 @@
     <xf numFmtId="177" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="178" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -547,9 +548,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="177" fontId="24" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="24" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
@@ -618,6 +616,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="24" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
@@ -996,17 +1003,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
       <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -1022,13 +1029,13 @@
       <c r="J2" s="13"/>
     </row>
     <row r="3" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
@@ -1036,13 +1043,13 @@
       <c r="J3" s="13"/>
     </row>
     <row r="4" spans="1:10" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="64" t="s">
+      <c r="A4" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="58"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
+      <c r="B4" s="55"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1050,13 +1057,13 @@
       <c r="J4" s="13"/>
     </row>
     <row r="5" spans="1:10" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="64" t="s">
+      <c r="A5" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="58"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
+      <c r="B5" s="55"/>
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
@@ -1076,35 +1083,35 @@
       <c r="J6" s="13"/>
     </row>
     <row r="7" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="67" t="s">
+      <c r="A7" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="67"/>
-      <c r="C7" s="63"/>
-      <c r="D7" s="63"/>
-      <c r="E7" s="63"/>
+      <c r="B7" s="64"/>
+      <c r="C7" s="60"/>
+      <c r="D7" s="60"/>
+      <c r="E7" s="60"/>
       <c r="F7" s="20"/>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63"/>
+      <c r="H7" s="60"/>
+      <c r="I7" s="60"/>
       <c r="J7" s="13"/>
     </row>
     <row r="8" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="68" t="s">
+      <c r="A8" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="68"/>
-      <c r="C8" s="55"/>
-      <c r="D8" s="55"/>
-      <c r="E8" s="55"/>
+      <c r="B8" s="65"/>
+      <c r="C8" s="52"/>
+      <c r="D8" s="52"/>
+      <c r="E8" s="52"/>
       <c r="F8" s="20"/>
-      <c r="G8" s="26" t="s">
+      <c r="G8" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H8" s="55"/>
-      <c r="I8" s="55"/>
+      <c r="H8" s="52"/>
+      <c r="I8" s="52"/>
       <c r="J8" s="13"/>
     </row>
     <row r="9" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1114,11 +1121,11 @@
       <c r="D9" s="19"/>
       <c r="E9" s="19"/>
       <c r="F9" s="20"/>
-      <c r="G9" s="26" t="s">
+      <c r="G9" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
+      <c r="H9" s="52"/>
+      <c r="I9" s="52"/>
       <c r="J9" s="13"/>
     </row>
     <row r="10" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1128,68 +1135,68 @@
       <c r="D10" s="19"/>
       <c r="E10" s="19"/>
       <c r="F10" s="20"/>
-      <c r="G10" s="26" t="s">
+      <c r="G10" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
+      <c r="H10" s="52"/>
+      <c r="I10" s="52"/>
       <c r="J10" s="13"/>
     </row>
     <row r="11" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="24" t="s">
         <v>19</v>
       </c>
       <c r="E11" s="17"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25" t="s">
+      <c r="F11" s="24"/>
+      <c r="G11" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="56"/>
-      <c r="I11" s="56"/>
+      <c r="H11" s="53"/>
+      <c r="I11" s="53"/>
       <c r="J11" s="13"/>
     </row>
     <row r="12" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="55"/>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
+      <c r="A12" s="52"/>
+      <c r="B12" s="52"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="52"/>
       <c r="F12" s="15"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="52"/>
+      <c r="I12" s="52"/>
       <c r="J12" s="13"/>
     </row>
     <row r="13" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="55"/>
-      <c r="B13" s="55"/>
-      <c r="C13" s="55"/>
-      <c r="D13" s="55"/>
-      <c r="E13" s="55"/>
+      <c r="A13" s="52"/>
+      <c r="B13" s="52"/>
+      <c r="C13" s="52"/>
+      <c r="D13" s="52"/>
+      <c r="E13" s="52"/>
       <c r="F13" s="15"/>
-      <c r="G13" s="55"/>
-      <c r="H13" s="55"/>
-      <c r="I13" s="55"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="52"/>
+      <c r="I13" s="52"/>
       <c r="J13" s="13"/>
     </row>
     <row r="14" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="55"/>
-      <c r="B14" s="55"/>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
+      <c r="A14" s="52"/>
+      <c r="B14" s="52"/>
+      <c r="C14" s="52"/>
+      <c r="D14" s="52"/>
+      <c r="E14" s="52"/>
       <c r="F14" s="15"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
+      <c r="G14" s="52"/>
+      <c r="H14" s="52"/>
+      <c r="I14" s="52"/>
       <c r="J14" s="13"/>
     </row>
     <row r="15" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="17"/>
-      <c r="B15" s="41"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="39"/>
       <c r="F15" s="15"/>
       <c r="G15" s="19"/>
       <c r="H15" s="15"/>
@@ -1197,118 +1204,118 @@
       <c r="J15" s="13"/>
     </row>
     <row r="16" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="69" t="s">
+      <c r="A16" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="70"/>
-      <c r="C16" s="70"/>
-      <c r="D16" s="70"/>
-      <c r="E16" s="29" t="s">
+      <c r="B16" s="67"/>
+      <c r="C16" s="67"/>
+      <c r="D16" s="67"/>
+      <c r="E16" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="30" t="s">
+      <c r="F16" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="G16" s="29" t="s">
+      <c r="G16" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="H16" s="65" t="s">
+      <c r="H16" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="I16" s="66"/>
+      <c r="I16" s="63"/>
       <c r="J16" s="13"/>
     </row>
     <row r="17" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="45"/>
-      <c r="B17" s="46"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="31"/>
-      <c r="I17" s="35"/>
+      <c r="A17" s="42"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="69"/>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="45"/>
-      <c r="B18" s="46"/>
-      <c r="C18" s="46"/>
-      <c r="D18" s="46"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="31"/>
-      <c r="I18" s="35"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="69"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="45"/>
-      <c r="B19" s="46"/>
-      <c r="C19" s="46"/>
-      <c r="D19" s="46"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="31"/>
-      <c r="I19" s="35"/>
+      <c r="A19" s="42"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="69"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="45"/>
-      <c r="B20" s="46"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="32"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="35"/>
+      <c r="A20" s="42"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="69"/>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="45"/>
-      <c r="B21" s="46"/>
-      <c r="C21" s="46"/>
-      <c r="D21" s="46"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="31"/>
-      <c r="I21" s="35"/>
+      <c r="A21" s="42"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="69"/>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="45"/>
-      <c r="B22" s="46"/>
-      <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="32"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="31"/>
-      <c r="I22" s="35"/>
+      <c r="A22" s="42"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="69"/>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="43"/>
-      <c r="B23" s="44"/>
-      <c r="C23" s="44"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="38"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="36"/>
-      <c r="I23" s="40"/>
+      <c r="A23" s="40"/>
+      <c r="B23" s="41"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="34"/>
+      <c r="I23" s="70"/>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="53" t="s">
+      <c r="A24" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="B24" s="54"/>
-      <c r="C24" s="54"/>
-      <c r="D24" s="54"/>
+      <c r="B24" s="51"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="51"/>
       <c r="E24" s="21">
         <f>SUM(E17:E23)</f>
         <v>0</v>
@@ -1316,24 +1323,24 @@
       <c r="F24" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G24" s="23"/>
+      <c r="G24" s="68"/>
       <c r="H24" s="22"/>
-      <c r="I24" s="24">
+      <c r="I24" s="23">
         <f>SUM(I17:I23)</f>
         <v>0</v>
       </c>
       <c r="J24" s="2"/>
     </row>
     <row r="25" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="51"/>
-      <c r="B25" s="52"/>
-      <c r="C25" s="52"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="52"/>
-      <c r="F25" s="52"/>
-      <c r="G25" s="52"/>
-      <c r="H25" s="52"/>
-      <c r="I25" s="52"/>
+      <c r="A25" s="48"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="49"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="49"/>
       <c r="J25" s="3"/>
     </row>
     <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1500,45 +1507,45 @@
       <c r="J39" s="6"/>
     </row>
     <row r="40" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="49" t="s">
+      <c r="A40" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="B40" s="50"/>
-      <c r="C40" s="50"/>
-      <c r="D40" s="50"/>
-      <c r="E40" s="50"/>
-      <c r="F40" s="50"/>
-      <c r="G40" s="50"/>
-      <c r="H40" s="50"/>
-      <c r="I40" s="50"/>
+      <c r="B40" s="47"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="47"/>
+      <c r="E40" s="47"/>
+      <c r="F40" s="47"/>
+      <c r="G40" s="47"/>
+      <c r="H40" s="47"/>
+      <c r="I40" s="47"/>
       <c r="J40" s="6"/>
     </row>
     <row r="41" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="27"/>
-      <c r="B41" s="28"/>
-      <c r="C41" s="28"/>
-      <c r="D41" s="28"/>
-      <c r="E41" s="28"/>
-      <c r="F41" s="28"/>
-      <c r="G41" s="28"/>
-      <c r="H41" s="28"/>
-      <c r="I41" s="28"/>
+      <c r="A41" s="26"/>
+      <c r="B41" s="27"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="27"/>
+      <c r="I41" s="27"/>
       <c r="J41" s="6"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A42" s="47" t="s">
+      <c r="A42" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="B42" s="48"/>
-      <c r="C42" s="48"/>
-      <c r="D42" s="48"/>
-      <c r="E42" s="48"/>
-      <c r="F42" s="57" t="s">
+      <c r="B42" s="45"/>
+      <c r="C42" s="45"/>
+      <c r="D42" s="45"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="G42" s="58"/>
-      <c r="H42" s="58"/>
-      <c r="I42" s="58"/>
+      <c r="G42" s="55"/>
+      <c r="H42" s="55"/>
+      <c r="I42" s="55"/>
       <c r="J42" s="7"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add FI generation by Customer PO — aggregate items across multiple DNs
When a purchase order spans multiple Delivery Notes, users can now generate
a single Final Invoice by entering the Customer PO number (e.g. 26KPO00144).
BAT menu updated with sub-menu for DN_ID vs Customer PO mode.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/final_invoice.xlsx
+++ b/templates/final_invoice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rotork-my.sharepoint.com/personal/jeongtaek_bang_rotork_com/Documents/바탕 화면/업무/NOAH ACTUATION/noahAutomation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{69FBBAE9-3359-454D-8387-2509559CBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCF52F5D-AEA5-43B5-8871-8C05B75C44BC}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="8_{69FBBAE9-3359-454D-8387-2509559CBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B79F06A-1FA2-41BD-A70D-5EA3A73E23C7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -449,7 +449,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -550,48 +550,15 @@
     <xf numFmtId="177" fontId="24" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="178" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="24" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -602,6 +569,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -612,18 +580,53 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="24" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1003,17 +1006,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
       <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -1029,13 +1032,13 @@
       <c r="J2" s="13"/>
     </row>
     <row r="3" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="58" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
@@ -1043,13 +1046,13 @@
       <c r="J3" s="13"/>
     </row>
     <row r="4" spans="1:10" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="61" t="s">
+      <c r="A4" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1057,13 +1060,13 @@
       <c r="J4" s="13"/>
     </row>
     <row r="5" spans="1:10" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="61" t="s">
+      <c r="A5" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="55"/>
-      <c r="C5" s="55"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
+      <c r="B5" s="47"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
@@ -1083,26 +1086,26 @@
       <c r="J6" s="13"/>
     </row>
     <row r="7" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="64" t="s">
+      <c r="A7" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="64"/>
-      <c r="C7" s="60"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="60"/>
+      <c r="B7" s="50"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="45"/>
       <c r="F7" s="20"/>
       <c r="G7" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="H7" s="60"/>
-      <c r="I7" s="60"/>
+      <c r="H7" s="45"/>
+      <c r="I7" s="45"/>
       <c r="J7" s="13"/>
     </row>
     <row r="8" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="65" t="s">
+      <c r="A8" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="65"/>
+      <c r="B8" s="51"/>
       <c r="C8" s="52"/>
       <c r="D8" s="52"/>
       <c r="E8" s="52"/>
@@ -1151,8 +1154,8 @@
       <c r="G11" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="53"/>
-      <c r="I11" s="53"/>
+      <c r="H11" s="55"/>
+      <c r="I11" s="55"/>
       <c r="J11" s="13"/>
     </row>
     <row r="12" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1193,10 +1196,10 @@
     </row>
     <row r="15" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="17"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
+      <c r="B15" s="57"/>
+      <c r="C15" s="58"/>
+      <c r="D15" s="58"/>
+      <c r="E15" s="58"/>
       <c r="F15" s="15"/>
       <c r="G15" s="19"/>
       <c r="H15" s="15"/>
@@ -1204,12 +1207,12 @@
       <c r="J15" s="13"/>
     </row>
     <row r="16" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="66" t="s">
+      <c r="A16" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="67"/>
-      <c r="C16" s="67"/>
-      <c r="D16" s="67"/>
+      <c r="B16" s="54"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="54"/>
       <c r="E16" s="28" t="s">
         <v>7</v>
       </c>
@@ -1219,111 +1222,111 @@
       <c r="G16" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="H16" s="62" t="s">
+      <c r="H16" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="I16" s="63"/>
+      <c r="I16" s="49"/>
       <c r="J16" s="13"/>
     </row>
     <row r="17" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="42"/>
-      <c r="B17" s="43"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
+      <c r="A17" s="67"/>
+      <c r="B17" s="68"/>
+      <c r="C17" s="68"/>
+      <c r="D17" s="68"/>
       <c r="E17" s="31"/>
       <c r="F17" s="32"/>
       <c r="G17" s="33"/>
       <c r="H17" s="30"/>
-      <c r="I17" s="69"/>
+      <c r="I17" s="39"/>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="42"/>
-      <c r="B18" s="43"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
+      <c r="A18" s="67"/>
+      <c r="B18" s="68"/>
+      <c r="C18" s="68"/>
+      <c r="D18" s="68"/>
       <c r="E18" s="31"/>
       <c r="F18" s="32"/>
       <c r="G18" s="33"/>
       <c r="H18" s="30"/>
-      <c r="I18" s="69"/>
+      <c r="I18" s="39"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="42"/>
-      <c r="B19" s="43"/>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
+      <c r="A19" s="67"/>
+      <c r="B19" s="68"/>
+      <c r="C19" s="68"/>
+      <c r="D19" s="68"/>
       <c r="E19" s="31"/>
       <c r="F19" s="32"/>
       <c r="G19" s="33"/>
       <c r="H19" s="30"/>
-      <c r="I19" s="69"/>
+      <c r="I19" s="39"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="42"/>
-      <c r="B20" s="43"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
+      <c r="A20" s="67"/>
+      <c r="B20" s="68"/>
+      <c r="C20" s="68"/>
+      <c r="D20" s="68"/>
       <c r="E20" s="31"/>
       <c r="F20" s="32"/>
       <c r="G20" s="33"/>
       <c r="H20" s="30"/>
-      <c r="I20" s="69"/>
+      <c r="I20" s="39"/>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="42"/>
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
+      <c r="A21" s="67"/>
+      <c r="B21" s="68"/>
+      <c r="C21" s="68"/>
+      <c r="D21" s="68"/>
       <c r="E21" s="31"/>
       <c r="F21" s="32"/>
       <c r="G21" s="33"/>
       <c r="H21" s="30"/>
-      <c r="I21" s="69"/>
+      <c r="I21" s="39"/>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="42"/>
-      <c r="B22" s="43"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
+      <c r="A22" s="67"/>
+      <c r="B22" s="68"/>
+      <c r="C22" s="68"/>
+      <c r="D22" s="68"/>
       <c r="E22" s="31"/>
       <c r="F22" s="32"/>
       <c r="G22" s="33"/>
       <c r="H22" s="30"/>
-      <c r="I22" s="69"/>
+      <c r="I22" s="39"/>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="40"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="41"/>
+      <c r="A23" s="69"/>
+      <c r="B23" s="70"/>
+      <c r="C23" s="70"/>
+      <c r="D23" s="70"/>
       <c r="E23" s="35"/>
       <c r="F23" s="36"/>
       <c r="G23" s="37"/>
       <c r="H23" s="34"/>
-      <c r="I23" s="70"/>
+      <c r="I23" s="40"/>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="50" t="s">
+      <c r="A24" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
+      <c r="B24" s="66"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="66"/>
       <c r="E24" s="21">
         <f>SUM(E17:E23)</f>
         <v>0</v>
       </c>
-      <c r="F24" s="22" t="s">
+      <c r="F24" s="71" t="s">
         <v>12</v>
       </c>
-      <c r="G24" s="68"/>
+      <c r="G24" s="38"/>
       <c r="H24" s="22"/>
       <c r="I24" s="23">
         <f>SUM(I17:I23)</f>
@@ -1332,15 +1335,15 @@
       <c r="J24" s="2"/>
     </row>
     <row r="25" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="48"/>
-      <c r="B25" s="49"/>
-      <c r="C25" s="49"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="49"/>
+      <c r="A25" s="63"/>
+      <c r="B25" s="64"/>
+      <c r="C25" s="64"/>
+      <c r="D25" s="64"/>
+      <c r="E25" s="64"/>
+      <c r="F25" s="64"/>
+      <c r="G25" s="64"/>
+      <c r="H25" s="64"/>
+      <c r="I25" s="64"/>
       <c r="J25" s="3"/>
     </row>
     <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1507,17 +1510,17 @@
       <c r="J39" s="6"/>
     </row>
     <row r="40" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="46" t="s">
+      <c r="A40" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="B40" s="47"/>
-      <c r="C40" s="47"/>
-      <c r="D40" s="47"/>
-      <c r="E40" s="47"/>
-      <c r="F40" s="47"/>
-      <c r="G40" s="47"/>
-      <c r="H40" s="47"/>
-      <c r="I40" s="47"/>
+      <c r="B40" s="62"/>
+      <c r="C40" s="62"/>
+      <c r="D40" s="62"/>
+      <c r="E40" s="62"/>
+      <c r="F40" s="62"/>
+      <c r="G40" s="62"/>
+      <c r="H40" s="62"/>
+      <c r="I40" s="62"/>
       <c r="J40" s="6"/>
     </row>
     <row r="41" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1533,23 +1536,39 @@
       <c r="J41" s="6"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A42" s="44" t="s">
+      <c r="A42" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="B42" s="45"/>
-      <c r="C42" s="45"/>
-      <c r="D42" s="45"/>
-      <c r="E42" s="45"/>
-      <c r="F42" s="54" t="s">
+      <c r="B42" s="60"/>
+      <c r="C42" s="60"/>
+      <c r="D42" s="60"/>
+      <c r="E42" s="60"/>
+      <c r="F42" s="56" t="s">
         <v>14</v>
       </c>
-      <c r="G42" s="55"/>
-      <c r="H42" s="55"/>
-      <c r="I42" s="55"/>
+      <c r="G42" s="47"/>
+      <c r="H42" s="47"/>
+      <c r="I42" s="47"/>
       <c r="J42" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="G12:I14"/>
+    <mergeCell ref="F42:I42"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="H7:I7"/>
@@ -1566,22 +1585,6 @@
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="G12:I14"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A42:E42"/>
-    <mergeCell ref="A40:I40"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A25:I25"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A20:D20"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <hyperlinks>

</xml_diff>